<commit_message>
docs: record third iteration experiment
</commit_message>
<xml_diff>
--- a/reports/蛋白质功能预测迭代趋势.xlsx
+++ b/reports/蛋白质功能预测迭代趋势.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="迭代趋势" sheetId="1" r:id="Re232f8f78be14cc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="迭代趋势" sheetId="1" r:id="R91814e2fe0b4442d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +18,7 @@
     <x:numFmt numFmtId="201" formatCode="0.000000"/>
     <x:numFmt numFmtId="202" formatCode="+0.000000;-0.000000;0.000000"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -72,8 +72,14 @@
       <x:sz val="11"/>
       <x:name val="Microsoft YaHei"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -115,8 +121,13 @@
         <x:fgColor rgb="FFD99A2B"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCE6ED"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="36">
+  <x:borders count="37">
     <x:border/>
     <x:border>
       <x:bottom style="medium">
@@ -404,11 +415,16 @@
         <x:color rgb="FFD99A2B"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFB4C6D4"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="176">
+  <x:cellXfs count="180">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -833,6 +849,12 @@
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -844,7 +866,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEA"/>
         </x:patternFill>
       </x:fill>
@@ -855,7 +877,7 @@
         <x:color rgb="FF137333"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE6F4EA"/>
         </x:patternFill>
       </x:fill>
@@ -1085,7 +1107,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R49c8923e9315414b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R78249e3eb7d64865"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1353,7 +1375,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="170" t="str">
-        <x:v>截至 2026-09-26｜主指标：Macro F1（越高越好）｜Macro AUC 作为辅助指标</x:v>
+        <x:v>每次迭代完成后更新｜截至 2026-09-26｜主指标：Macro F1（越高越好）｜Macro AUC 作为辅助指标</x:v>
       </x:c>
       <x:c r="B3" s="174"/>
       <x:c r="C3" s="174"/>
@@ -1947,7 +1969,7 @@
     </x:row>
     <x:row r="24" ht="26" customHeight="1">
       <x:c r="A24" s="126" t="str">
-        <x:v>第一次：EXP-20260923-025；第二次：EXP-20260924-030；第三次：EXP-20260926-044/045。</x:v>
+        <x:v>第一次：EXP-20260923-025；第二次：EXP-20260924-030；第三次：EXP-20260926-iteration3（实验编号 EXP-20260926-044/045）。</x:v>
       </x:c>
       <x:c r="B24" s="126"/>
       <x:c r="C24" s="126"/>
@@ -1968,7 +1990,7 @@
     </x:row>
     <x:row r="25" ht="26" customHeight="1">
       <x:c r="A25" s="126" t="str">
-        <x:v>来源：各轮实验报告、阈值摘要 JSON 与第三次实验最终报告。</x:v>
+        <x:v>来源：各轮独立实验报告、阈值摘要 JSON 与迭代完成后的提交校验记录。</x:v>
       </x:c>
       <x:c r="B25" s="126"/>
       <x:c r="C25" s="126"/>
@@ -1987,6 +2009,66 @@
       <x:c r="P25" s="174"/>
       <x:c r="Q25" s="174"/>
     </x:row>
+    <x:row r="27" ht="24" customHeight="1">
+      <x:c r="A27" s="179" t="str">
+        <x:v>迭代表更新规则</x:v>
+      </x:c>
+      <x:c r="B27" s="179"/>
+      <x:c r="C27" s="179"/>
+      <x:c r="D27" s="179"/>
+      <x:c r="E27" s="179"/>
+      <x:c r="F27" s="179"/>
+      <x:c r="G27" s="179"/>
+      <x:c r="H27" s="179"/>
+    </x:row>
+    <x:row r="28" ht="24" customHeight="1">
+      <x:c r="A28" t="str">
+        <x:v>1. 只登记已经完成的迭代。</x:v>
+      </x:c>
+      <x:c r="B28"/>
+      <x:c r="C28"/>
+      <x:c r="D28"/>
+      <x:c r="E28"/>
+      <x:c r="F28"/>
+      <x:c r="G28"/>
+      <x:c r="H28"/>
+    </x:row>
+    <x:row r="29" ht="24" customHeight="1">
+      <x:c r="A29" t="str">
+        <x:v>2. 每轮完成独立实验报告后，在上方迭代表新增一行。</x:v>
+      </x:c>
+      <x:c r="B29"/>
+      <x:c r="C29"/>
+      <x:c r="D29"/>
+      <x:c r="E29"/>
+      <x:c r="F29"/>
+      <x:c r="G29"/>
+      <x:c r="H29"/>
+    </x:row>
+    <x:row r="30" ht="24" customHeight="1">
+      <x:c r="A30" t="str">
+        <x:v>3. 每轮记录验证口径、Macro F1、Macro AUC、结论和报告编号。</x:v>
+      </x:c>
+      <x:c r="B30"/>
+      <x:c r="C30"/>
+      <x:c r="D30"/>
+      <x:c r="E30"/>
+      <x:c r="F30"/>
+      <x:c r="G30"/>
+      <x:c r="H30"/>
+    </x:row>
+    <x:row r="31" ht="24" customHeight="1">
+      <x:c r="A31" t="str">
+        <x:v>4. 最终综合报告在全部迭代结束后再编写。</x:v>
+      </x:c>
+      <x:c r="B31"/>
+      <x:c r="C31"/>
+      <x:c r="D31"/>
+      <x:c r="E31"/>
+      <x:c r="F31"/>
+      <x:c r="G31"/>
+      <x:c r="H31"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A18:H19"/>
@@ -1995,6 +2077,11 @@
     <x:mergeCell ref="A25:H25"/>
     <x:mergeCell ref="J17:Q17"/>
     <x:mergeCell ref="J18:Q20"/>
+    <x:mergeCell ref="A27:H27"/>
+    <x:mergeCell ref="A28:H28"/>
+    <x:mergeCell ref="A29:H29"/>
+    <x:mergeCell ref="A30:H30"/>
+    <x:mergeCell ref="A31:H31"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B12:B14">
     <x:cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
@@ -2005,6 +2092,6 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6aae614265c4a00"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R863761212bbb4a7f"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add iteration 5 homology blend submission pipeline
</commit_message>
<xml_diff>
--- a/reports/蛋白质功能预测迭代趋势.xlsx
+++ b/reports/蛋白质功能预测迭代趋势.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="迭代趋势" sheetId="1" r:id="R91814e2fe0b4442d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="迭代趋势" sheetId="1" r:id="R91fb7c4566a14e68"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -933,20 +933,12 @@
           <c:tx>
             <c:v>Macro F1</c:v>
           </c:tx>
-          <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575">
-              <a:solidFill>
-                <a:srgbClr val="2F6B8A"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'迭代趋势'!$A$6:$A$8</c:f>
+              <c:f>'迭代趋势'!$A$6:$A$10</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -954,7 +946,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'迭代趋势'!$E$6:$E$8</c:f>
+              <c:f>'迭代趋势'!$E$6:$E$10</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1107,7 +1099,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R78249e3eb7d64865"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9856331aa2cc41c8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1375,7 +1367,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="170" t="str">
-        <x:v>每次迭代完成后更新｜截至 2026-09-26｜主指标：Macro F1（越高越好）｜Macro AUC 作为辅助指标</x:v>
+        <x:v>每次迭代完成后更新｜截至 2026-09-28｜主指标：Macro F1（越高越好）｜Macro AUC 作为辅助指标</x:v>
       </x:c>
       <x:c r="B3" s="174"/>
       <x:c r="C3" s="174"/>
@@ -1553,15 +1545,31 @@
       <x:c r="P8" s="174"/>
       <x:c r="Q8" s="174"/>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="174"/>
-      <x:c r="B9" s="174"/>
-      <x:c r="C9" s="174"/>
-      <x:c r="D9" s="174"/>
-      <x:c r="E9" s="174"/>
-      <x:c r="F9" s="174"/>
-      <x:c r="G9" s="174"/>
-      <x:c r="H9" s="174"/>
+    <x:row r="9" ht="56" customHeight="1">
+      <x:c r="A9" s="67" t="str">
+        <x:v>第四次</x:v>
+      </x:c>
+      <x:c r="B9" s="68" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="C9" s="69" t="str">
+        <x:v>SGD/KNN 60% + GPU CNN 40%（固定 8 epoch）</x:v>
+      </x:c>
+      <x:c r="D9" s="69" t="str">
+        <x:v>尾段代理验证（1,062 样本，5 个 threshold split seeds）</x:v>
+      </x:c>
+      <x:c r="E9" s="70" t="n">
+        <x:v>0.32419172996031437</x:v>
+      </x:c>
+      <x:c r="F9" s="71" t="n">
+        <x:v>0.0012013940043014708</x:v>
+      </x:c>
+      <x:c r="G9" s="71" t="n">
+        <x:v>0.8280390455031759</x:v>
+      </x:c>
+      <x:c r="H9" s="69" t="str">
+        <x:v>同口径 F1 +0.002675；AUC +0.012994，未达到 0.5</x:v>
+      </x:c>
       <x:c r="I9" s="174"/>
       <x:c r="J9" s="174"/>
       <x:c r="K9" s="174"/>
@@ -1572,15 +1580,31 @@
       <x:c r="P9" s="174"/>
       <x:c r="Q9" s="174"/>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="174"/>
-      <x:c r="B10" s="174"/>
-      <x:c r="C10" s="174"/>
-      <x:c r="D10" s="174"/>
-      <x:c r="E10" s="174"/>
-      <x:c r="F10" s="174"/>
-      <x:c r="G10" s="174"/>
-      <x:c r="H10" s="174"/>
+    <x:row r="10" ht="56" customHeight="1">
+      <x:c r="A10" s="67" t="str">
+        <x:v>第五次</x:v>
+      </x:c>
+      <x:c r="B10" s="68" t="n">
+        <x:v>46293</x:v>
+      </x:c>
+      <x:c r="C10" s="69" t="str">
+        <x:v>序列局部对齐近邻 90% + 尾段加权 SGD 10%</x:v>
+      </x:c>
+      <x:c r="D10" s="69" t="str">
+        <x:v>尾段代理验证（1,062 样本，5 个 threshold split seeds）</x:v>
+      </x:c>
+      <x:c r="E10" s="70" t="n">
+        <x:v>0.3351783934801672</x:v>
+      </x:c>
+      <x:c r="F10" s="71" t="n">
+        <x:v>0.0008049006706986432</x:v>
+      </x:c>
+      <x:c r="G10" s="71" t="n">
+        <x:v>0.8211324963363611</x:v>
+      </x:c>
+      <x:c r="H10" s="69" t="str">
+        <x:v>F1 +0.010987；AUC 高于第三次但低于第四次</x:v>
+      </x:c>
       <x:c r="I10" s="174"/>
       <x:c r="J10" s="174"/>
       <x:c r="K10" s="174"/>
@@ -1694,10 +1718,17 @@
       <x:c r="P14" s="174"/>
       <x:c r="Q14" s="174"/>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="174"/>
-      <x:c r="B15" s="174"/>
-      <x:c r="C15" s="174"/>
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="88" t="str">
+        <x:v>第三次 → 第四次</x:v>
+      </x:c>
+      <x:c r="B15" s="94" t="n">
+        <x:f>E9-E8</x:f>
+        <x:v>0.0026748030171062642</x:v>
+      </x:c>
+      <x:c r="C15" s="97" t="str">
+        <x:v>同口径：尾段五 seed F1 小幅提升；AUC 同时提高</x:v>
+      </x:c>
       <x:c r="D15" s="174"/>
       <x:c r="E15" s="174"/>
       <x:c r="F15" s="174"/>
@@ -1714,9 +1745,16 @@
       <x:c r="Q15" s="174"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="174"/>
-      <x:c r="B16" s="174"/>
-      <x:c r="C16" s="174"/>
+      <x:c r="A16" s="88" t="str">
+        <x:v>第四次 → 第五次</x:v>
+      </x:c>
+      <x:c r="B16" s="94" t="n">
+        <x:f>E10-E9</x:f>
+        <x:v>0.010986663519852835</x:v>
+      </x:c>
+      <x:c r="C16" s="97" t="str">
+        <x:v>同口径：局部对齐提高 F1；AUC 相对第四次回落</x:v>
+      </x:c>
       <x:c r="D16" s="174"/>
       <x:c r="E16" s="174"/>
       <x:c r="F16" s="174"/>
@@ -1771,7 +1809,7 @@
     </x:row>
     <x:row r="18" ht="32" customHeight="1">
       <x:c r="A18" s="115" t="str">
-        <x:v>第三次迭代采用更接近测试 ID 分布的尾段代理验证，前两次采用固定随机验证。折线图展示各轮本地代表指标及方法演进，不表示严格同口径的绝对升降。前两轮现有指标文件未记录连续 Macro AUC，因此保留为“未记录”，不以 0 代替。</x:v>
+        <x:v>第三、四次采用相同尾段代理验证和五个 threshold split seeds，可在两轮之间比较。前两次采用固定随机验证，不能与尾段结果直接比较。前两轮未记录连续 Macro AUC，保留为“未记录”。</x:v>
       </x:c>
       <x:c r="B18" s="116" t="str">
         <x:v>第三次迭代采用更接近测试 ID 分布的尾段代理验证，前两次采用固定随机验证。折线图展示各轮本地代表指标及方法演进，不表示严格同口径的绝对升降。前两轮现有指标文件未记录连续 Macro AUC，因此保留为“未记录”，不以 0 代替。</x:v>
@@ -1796,7 +1834,7 @@
       </x:c>
       <x:c r="I18" s="174"/>
       <x:c r="J18" s="159" t="str">
-        <x:v>第三次数据点使用尾段代理验证。结合方法变化和验证口径阅读，不把折线斜率直接解释为线上成绩升降。</x:v>
+        <x:v>前两次与后两次验证口径不同；第三次到第四次同口径。折线图展示本地代理指标，不代表平台实际得分。</x:v>
       </x:c>
       <x:c r="K18" s="160" t="str">
         <x:v>第三次数据点使用尾段代理验证。结合方法变化和验证口径阅读，不把折线斜率直接解释为线上成绩升降。</x:v>
@@ -1872,7 +1910,9 @@
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="174"/>
+      <x:c r="A20" s="174" t="str">
+        <x:v>第三、四、五次采用相同尾段代理验证和五个 threshold split seeds，可在三轮之间比较。前两次采用固定随机验证，不能与尾段结果直接比较。前两轮未记录连续 Macro AUC，保留为“未记录”。</x:v>
+      </x:c>
       <x:c r="B20" s="174"/>
       <x:c r="C20" s="174"/>
       <x:c r="D20" s="174"/>
@@ -1882,7 +1922,7 @@
       <x:c r="H20" s="174"/>
       <x:c r="I20" s="174"/>
       <x:c r="J20" s="165" t="str">
-        <x:v>第三次数据点使用尾段代理验证。结合方法变化和验证口径阅读，不把折线斜率直接解释为线上成绩升降。</x:v>
+        <x:v>前两次与后三次验证口径不同；第三次到第五次为同口径。折线图展示本地代理指标，不代表平台实际得分。</x:v>
       </x:c>
       <x:c r="K20" s="166" t="str">
         <x:v>第三次数据点使用尾段代理验证。结合方法变化和验证口径阅读，不把折线斜率直接解释为线上成绩升降。</x:v>
@@ -1969,7 +2009,7 @@
     </x:row>
     <x:row r="24" ht="26" customHeight="1">
       <x:c r="A24" s="126" t="str">
-        <x:v>第一次：EXP-20260923-025；第二次：EXP-20260924-030；第三次：EXP-20260926-iteration3（实验编号 EXP-20260926-044/045）。</x:v>
+        <x:v>第一次：EXP-20260923-025；第二次：EXP-20260924-030；第三次：EXP-20260926-044/045；第四次：EXP-20260928-065；第五次：EXP-20260928-068/070。</x:v>
       </x:c>
       <x:c r="B24" s="126"/>
       <x:c r="C24" s="126"/>
@@ -2092,6 +2132,6 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R863761212bbb4a7f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re002bfecfc884ee6"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add iteration7 labelwise search and run artifacts
</commit_message>
<xml_diff>
--- a/reports/蛋白质功能预测迭代趋势.xlsx
+++ b/reports/蛋白质功能预测迭代趋势.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="迭代趋势" sheetId="1" r:id="R91fb7c4566a14e68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="迭代趋势" sheetId="1" r:id="R9bf9588a2e2f422c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -938,7 +938,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'迭代趋势'!$A$6:$A$10</c:f>
+              <c:f>'迭代趋势'!$A$6:$A$11</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -946,7 +946,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'迭代趋势'!$E$6:$E$10</c:f>
+              <c:f>'迭代趋势'!$E$6:$E$11</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1099,7 +1099,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9856331aa2cc41c8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R552928d58132466a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1367,7 +1367,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="170" t="str">
-        <x:v>每次迭代完成后更新｜截至 2026-09-28｜主指标：Macro F1（越高越好）｜Macro AUC 作为辅助指标</x:v>
+        <x:v>每次迭代完成后更新｜截至 2026-09-29｜主指标：本地 Macro F1（越高越好）｜Macro AUC 作为辅助指标</x:v>
       </x:c>
       <x:c r="B3" s="174"/>
       <x:c r="C3" s="174"/>
@@ -1615,21 +1615,31 @@
       <x:c r="P10" s="174"/>
       <x:c r="Q10" s="174"/>
     </x:row>
-    <x:row r="11" ht="28" customHeight="1">
-      <x:c r="A11" s="76" t="str">
-        <x:v>对比</x:v>
-      </x:c>
-      <x:c r="B11" s="76" t="str">
-        <x:v>Macro F1 数值变化</x:v>
-      </x:c>
-      <x:c r="C11" s="76" t="str">
-        <x:v>解读</x:v>
-      </x:c>
-      <x:c r="D11" s="174"/>
-      <x:c r="E11" s="174"/>
-      <x:c r="F11" s="174"/>
-      <x:c r="G11" s="174"/>
-      <x:c r="H11" s="174"/>
+    <x:row r="11" ht="56" customHeight="1">
+      <x:c r="A11" s="67" t="str">
+        <x:v>第六次</x:v>
+      </x:c>
+      <x:c r="B11" s="68" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="C11" s="69" t="str">
+        <x:v>冻结 ESM-2 表示 + 按标签分类/融合（089 自适应候选）</x:v>
+      </x:c>
+      <x:c r="D11" s="69" t="str">
+        <x:v>尾段代理验证（1,062 样本，5 个 threshold split seeds）</x:v>
+      </x:c>
+      <x:c r="E11" s="70" t="n">
+        <x:v>0.3242434409979672</x:v>
+      </x:c>
+      <x:c r="F11" s="71" t="n">
+        <x:v>0.013719475982240131</x:v>
+      </x:c>
+      <x:c r="G11" s="71" t="n">
+        <x:v>0.8281240938209207</x:v>
+      </x:c>
+      <x:c r="H11" s="69" t="str">
+        <x:v>未超过第五次 F1；ESM 未入选策略；未生成新平台提交</x:v>
+      </x:c>
       <x:c r="I11" s="174"/>
       <x:c r="J11" s="174"/>
       <x:c r="K11" s="174"/>
@@ -1641,15 +1651,14 @@
       <x:c r="Q11" s="174"/>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
-      <x:c r="A12" s="86" t="str">
-        <x:v>第一次 → 第二次</x:v>
-      </x:c>
-      <x:c r="B12" s="92" t="n">
-        <x:f>E7-E6</x:f>
-        <x:v>-0.1335869304474091</x:v>
-      </x:c>
-      <x:c r="C12" s="95" t="str">
-        <x:v>同口径：GPU CNN 未超过 TF-IDF + SGD</x:v>
+      <x:c r="A12" s="76" t="str">
+        <x:v>对比</x:v>
+      </x:c>
+      <x:c r="B12" s="76" t="str">
+        <x:v>Macro F1 数值变化</x:v>
+      </x:c>
+      <x:c r="C12" s="76" t="str">
+        <x:v>解读</x:v>
       </x:c>
       <x:c r="D12" s="174"/>
       <x:c r="E12" s="174"/>
@@ -1667,15 +1676,15 @@
       <x:c r="Q12" s="174"/>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
-      <x:c r="A13" s="87" t="str">
-        <x:v>第二次 → 第三次</x:v>
-      </x:c>
-      <x:c r="B13" s="93" t="n">
-        <x:f>E8-E7</x:f>
-        <x:v>0.07514736443238412</x:v>
-      </x:c>
-      <x:c r="C13" s="96" t="str">
-        <x:v>不同口径：数值回升，但不可视为严格同比</x:v>
+      <x:c r="A13" s="86" t="str">
+        <x:v>第一次 → 第二次</x:v>
+      </x:c>
+      <x:c r="B13" s="92" t="n">
+        <x:f>E7-E6</x:f>
+        <x:v>-0.1335869304474091</x:v>
+      </x:c>
+      <x:c r="C13" s="95" t="str">
+        <x:v>同口径：GPU CNN 未超过 TF-IDF + SGD</x:v>
       </x:c>
       <x:c r="D13" s="174"/>
       <x:c r="E13" s="174"/>
@@ -1693,15 +1702,15 @@
       <x:c r="Q13" s="174"/>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
-      <x:c r="A14" s="88" t="str">
-        <x:v>第一次 → 第三次</x:v>
-      </x:c>
-      <x:c r="B14" s="94" t="n">
-        <x:f>E8-E6</x:f>
-        <x:v>-0.05843956601502498</x:v>
-      </x:c>
-      <x:c r="C14" s="97" t="str">
-        <x:v>不同口径：第三次更贴近测试 ID 分布</x:v>
+      <x:c r="A14" s="87" t="str">
+        <x:v>第二次 → 第三次</x:v>
+      </x:c>
+      <x:c r="B14" s="93" t="n">
+        <x:f>E8-E7</x:f>
+        <x:v>0.07514736443238412</x:v>
+      </x:c>
+      <x:c r="C14" s="96" t="str">
+        <x:v>不同口径：数值回升，但不可视为严格同比</x:v>
       </x:c>
       <x:c r="D14" s="174"/>
       <x:c r="E14" s="174"/>
@@ -1771,16 +1780,21 @@
       <x:c r="Q16" s="174"/>
     </x:row>
     <x:row r="17" ht="26" customHeight="1">
-      <x:c r="A17" s="172" t="str">
-        <x:v>验证口径说明</x:v>
-      </x:c>
-      <x:c r="B17" s="172"/>
-      <x:c r="C17" s="172"/>
-      <x:c r="D17" s="172"/>
-      <x:c r="E17" s="172"/>
-      <x:c r="F17" s="172"/>
-      <x:c r="G17" s="172"/>
-      <x:c r="H17" s="172"/>
+      <x:c r="A17" s="88" t="str">
+        <x:v>第五次 → 第六次</x:v>
+      </x:c>
+      <x:c r="B17" s="94" t="n">
+        <x:f>E11-E10</x:f>
+        <x:v>-0.0109349524822</x:v>
+      </x:c>
+      <x:c r="C17" s="97" t="str">
+        <x:v>同口径：标签自适应候选 F1 回落；AUC 小幅上升，未生成提交</x:v>
+      </x:c>
+      <x:c r="D17" s="174"/>
+      <x:c r="E17" s="174"/>
+      <x:c r="F17" s="174"/>
+      <x:c r="G17" s="174"/>
+      <x:c r="H17" s="174"/>
       <x:c r="I17" s="174"/>
       <x:c r="J17" s="130" t="str">
         <x:v>阅读提示</x:v>
@@ -1809,7 +1823,7 @@
     </x:row>
     <x:row r="18" ht="32" customHeight="1">
       <x:c r="A18" s="115" t="str">
-        <x:v>第三、四次采用相同尾段代理验证和五个 threshold split seeds，可在两轮之间比较。前两次采用固定随机验证，不能与尾段结果直接比较。前两轮未记录连续 Macro AUC，保留为“未记录”。</x:v>
+        <x:v>验证口径说明：第三至第六次均采用尾段代理验证和五个 threshold split seeds，可比较本地结果。前两次为固定随机验证，不可直接同比；第六次没有平台提交。第五次平台反馈：F1 0.379829、AUC 0.720675，与本地代理不同。</x:v>
       </x:c>
       <x:c r="B18" s="116" t="str">
         <x:v>第三次迭代采用更接近测试 ID 分布的尾段代理验证，前两次采用固定随机验证。折线图展示各轮本地代表指标及方法演进，不表示严格同口径的绝对升降。前两轮现有指标文件未记录连续 Macro AUC，因此保留为“未记录”，不以 0 代替。</x:v>
@@ -1834,7 +1848,7 @@
       </x:c>
       <x:c r="I18" s="174"/>
       <x:c r="J18" s="159" t="str">
-        <x:v>前两次与后两次验证口径不同；第三次到第四次同口径。折线图展示本地代理指标，不代表平台实际得分。</x:v>
+        <x:v>前两次与后四次验证口径不同；第三次到第六次可同口径比较本地代理结果。折线图不代表平台实际得分。第五次平台 F1 为 0.379829，AUC 为 0.720675。</x:v>
       </x:c>
       <x:c r="K18" s="160" t="str">
         <x:v>第三次数据点使用尾段代理验证。结合方法变化和验证口径阅读，不把折线斜率直接解释为线上成绩升降。</x:v>
@@ -2009,7 +2023,7 @@
     </x:row>
     <x:row r="24" ht="26" customHeight="1">
       <x:c r="A24" s="126" t="str">
-        <x:v>第一次：EXP-20260923-025；第二次：EXP-20260924-030；第三次：EXP-20260926-044/045；第四次：EXP-20260928-065；第五次：EXP-20260928-068/070。</x:v>
+        <x:v>第一次：EXP-20260923-025；第二次：EXP-20260924-030；第三次：EXP-20260926-044/045；第四次：EXP-20260928-065；第五次：EXP-20260928-068/070；第六次：EXP-20260929-089。</x:v>
       </x:c>
       <x:c r="B24" s="126"/>
       <x:c r="C24" s="126"/>
@@ -2132,6 +2146,6 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re002bfecfc884ee6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcdd2184a9564565"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
exp: report EXP-125 epoch slopes and reproducible ESM training
</commit_message>
<xml_diff>
--- a/reports/蛋白质功能预测迭代趋势.xlsx
+++ b/reports/蛋白质功能预测迭代趋势.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="迭代趋势" sheetId="1" r:id="R9bf9588a2e2f422c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="迭代趋势" sheetId="1" r:id="Rdd1ed17895b94b79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="趋势图数据" sheetId="2" r:id="R1be3ec92dfa448f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +19,7 @@
     <x:numFmt numFmtId="201" formatCode="0.000000"/>
     <x:numFmt numFmtId="202" formatCode="+0.000000;-0.000000;0.000000"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -78,8 +79,13 @@
       <x:color rgb="FF17365D"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -126,6 +132,31 @@
         <x:fgColor rgb="FFDCE6ED"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="37">
     <x:border/>
@@ -424,7 +455,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="180">
+  <x:cellXfs count="191">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -855,6 +886,25 @@
     <x:xf numFmtId="0" fontId="10" fillId="9" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -898,12 +948,12 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:rPr sz="975">
+              <a:rPr sz="1050">
                 <a:latin typeface="Microsoft YaHei"/>
                 <a:ea typeface="Microsoft YaHei"/>
                 <a:cs typeface="Microsoft YaHei"/>
               </a:rPr>
-              <a:t>各次迭代 Macro F1</a:t>
+              <a:t>500 标签尾段 Macro F1（目标 0.5）</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -914,7 +964,7 @@
         <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="975">
+            <a:defRPr sz="1050">
               <a:latin typeface="Microsoft YaHei"/>
               <a:ea typeface="Microsoft YaHei"/>
               <a:cs typeface="Microsoft YaHei"/>
@@ -933,12 +983,23 @@
           <c:tx>
             <c:v>Macro F1</c:v>
           </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="1F4E78"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="1F4E78"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'迭代趋势'!$A$6:$A$11</c:f>
+              <c:f>'趋势图数据'!$A$5:$A$15</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -946,7 +1007,233 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'迭代趋势'!$E$6:$E$11</c:f>
+              <c:f>'趋势图数据'!$B$5:$B$15</c:f>
+              <c:numCache>
+                <c:formatCode>0.000000</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>目标 0.5</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="C0504D"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="C0504D"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'趋势图数据'!$A$5:$A$15</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'趋势图数据'!$C$5:$C$15</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:smooth val="0"/>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="825">
+                <a:latin typeface="Microsoft YaHei"/>
+                <a:ea typeface="Microsoft YaHei"/>
+                <a:cs typeface="Microsoft YaHei"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.000" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr>
+                <a:latin typeface="Microsoft YaHei"/>
+                <a:ea typeface="Microsoft YaHei"/>
+                <a:cs typeface="Microsoft YaHei"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="825">
+              <a:latin typeface="Microsoft YaHei"/>
+              <a:ea typeface="Microsoft YaHei"/>
+              <a:cs typeface="Microsoft YaHei"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:rPr sz="1050">
+                <a:latin typeface="Microsoft YaHei"/>
+                <a:ea typeface="Microsoft YaHei"/>
+                <a:cs typeface="Microsoft YaHei"/>
+              </a:rPr>
+              <a:t>100 标签筛选 Macro F1（非全量成绩）</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="1050">
+              <a:latin typeface="Microsoft YaHei"/>
+              <a:ea typeface="Microsoft YaHei"/>
+              <a:cs typeface="Microsoft YaHei"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:plotArea>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Macro F1</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="548235"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="548235"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'趋势图数据'!$E$5:$E$8</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'趋势图数据'!$F$5:$F$8</c:f>
               <c:numCache>
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="0"/>
@@ -976,20 +1263,6 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:r>
-                  <a:t>迭代</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-        </c:title>
         <c:numFmt formatCode="General"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -999,7 +1272,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="750">
+              <a:defRPr sz="825">
                 <a:latin typeface="Microsoft YaHei"/>
                 <a:ea typeface="Microsoft YaHei"/>
                 <a:cs typeface="Microsoft YaHei"/>
@@ -1026,20 +1299,6 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:r>
-                  <a:t>Macro F1</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-        </c:title>
         <c:numFmt formatCode="0.000" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1048,7 +1307,177 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="750">
+              <a:defRPr>
+                <a:latin typeface="Microsoft YaHei"/>
+                <a:ea typeface="Microsoft YaHei"/>
+                <a:cs typeface="Microsoft YaHei"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48650112"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:r>
+              <a:rPr sz="1050">
+                <a:latin typeface="Microsoft YaHei"/>
+                <a:ea typeface="Microsoft YaHei"/>
+                <a:cs typeface="Microsoft YaHei"/>
+              </a:rPr>
+              <a:t>历史随机验证 Macro F1（不同口径）</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="1050">
+              <a:latin typeface="Microsoft YaHei"/>
+              <a:ea typeface="Microsoft YaHei"/>
+              <a:cs typeface="Microsoft YaHei"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:plotArea>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Macro F1</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="7F7F7F"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="7F7F7F"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'趋势图数据'!$H$5:$H$6</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'趋势图数据'!$I$5:$I$6</c:f>
+              <c:numCache>
+                <c:formatCode>0.000000</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:smooth val="0"/>
+        <c:axId val="48650112"/>
+        <c:axId val="48672768"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="48650112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="825">
+                <a:latin typeface="Microsoft YaHei"/>
+                <a:ea typeface="Microsoft YaHei"/>
+                <a:cs typeface="Microsoft YaHei"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48672768"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48672768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.000" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr>
                 <a:latin typeface="Microsoft YaHei"/>
                 <a:ea typeface="Microsoft YaHei"/>
                 <a:cs typeface="Microsoft YaHei"/>
@@ -1085,7 +1514,7 @@
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1099,7 +1528,67 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R552928d58132466a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdc711628daa14394"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbfc8d82a06c04fc5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
+        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R79d021ef5fe841d5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1367,7 +1856,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="170" t="str">
-        <x:v>每次迭代完成后更新｜截至 2026-09-29｜主指标：本地 Macro F1（越高越好）｜Macro AUC 作为辅助指标</x:v>
+        <x:v>每次迭代完成后更新｜截至 2026-09-30｜主指标：本地 Macro F1（越高越好）｜Macro AUC 作为辅助指标</x:v>
       </x:c>
       <x:c r="B3" s="174"/>
       <x:c r="C3" s="174"/>
@@ -2122,6 +2611,323 @@
       <x:c r="F31"/>
       <x:c r="G31"/>
       <x:c r="H31"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="180" t="str">
+        <x:v>后续已完成迭代</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="15" t="str">
+        <x:v>迭代</x:v>
+      </x:c>
+      <x:c r="B34" s="16" t="str">
+        <x:v>日期</x:v>
+      </x:c>
+      <x:c r="C34" s="16" t="str">
+        <x:v>核心方案</x:v>
+      </x:c>
+      <x:c r="D34" s="16" t="str">
+        <x:v>验证口径</x:v>
+      </x:c>
+      <x:c r="E34" s="16" t="str">
+        <x:v>Macro F1</x:v>
+      </x:c>
+      <x:c r="F34" s="16" t="str">
+        <x:v>F1 标准差</x:v>
+      </x:c>
+      <x:c r="G34" s="16" t="str">
+        <x:v>Macro AUC</x:v>
+      </x:c>
+      <x:c r="H34" s="17" t="str">
+        <x:v>主要结论</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="90" customHeight="1">
+      <x:c r="A35" s="181" t="str">
+        <x:v>第七次（产物复核）</x:v>
+      </x:c>
+      <x:c r="B35" s="182" t="d">
+        <x:v>2026-09-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C35" s="69" t="str">
+        <x:v>标签级融合筛选：当前 EXP-095 自适应产物</x:v>
+      </x:c>
+      <x:c r="D35" s="69" t="str">
+        <x:v>尾段 1,062 样本、500 标签；原产物五 seed 汇总</x:v>
+      </x:c>
+      <x:c r="E35" s="183" t="n">
+        <x:v>0.32430998512037634</x:v>
+      </x:c>
+      <x:c r="F35" s="184" t="n">
+        <x:v>0.013956042497509615</x:v>
+      </x:c>
+      <x:c r="G35" s="184" t="n">
+        <x:v>0.8280838467649557</x:v>
+      </x:c>
+      <x:c r="H35" s="69" t="str">
+        <x:v>与原报告快照不一致，已加审计注释；不替换回退。报告：iteration7-labelwise-weighted</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="90" customHeight="1">
+      <x:c r="A36" s="181" t="str">
+        <x:v>第八次</x:v>
+      </x:c>
+      <x:c r="B36" s="182" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C36" s="69" t="str">
+        <x:v>25% ESM + 75% 同源/SGD，精确收缩阈值</x:v>
+      </x:c>
+      <x:c r="D36" s="69" t="str">
+        <x:v>固定尾段 1,062 样本、500 标签；五 seed 两折合并</x:v>
+      </x:c>
+      <x:c r="E36" s="183" t="n">
+        <x:v>0.3382479496821853</x:v>
+      </x:c>
+      <x:c r="F36" s="184" t="n">
+        <x:v>0.0010220441855182344</x:v>
+      </x:c>
+      <x:c r="G36" s="184" t="n">
+        <x:v>0.8244919055304825</x:v>
+      </x:c>
+      <x:c r="H36" s="69" t="str">
+        <x:v>EXP-103 为现有完整标签回退；未达到 0.5。报告：iteration8-rank-fusion</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="90" customHeight="1">
+      <x:c r="A37" s="181" t="str">
+        <x:v>联合特征筛选（111）</x:v>
+      </x:c>
+      <x:c r="B37" s="182" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C37" s="69" t="str">
+        <x:v>k-mer + 0.1 倍 ESM 表征联合 SGD</x:v>
+      </x:c>
+      <x:c r="D37" s="69" t="str">
+        <x:v>固定尾段 1,062 样本、支持度分层 100 标签；五 seed</x:v>
+      </x:c>
+      <x:c r="E37" s="183" t="n">
+        <x:v>0.3184272015000932</x:v>
+      </x:c>
+      <x:c r="F37" s="184" t="n">
+        <x:v>0.001091803390844629</x:v>
+      </x:c>
+      <x:c r="G37" s="184" t="n">
+        <x:v>0.8091421014599195</x:v>
+      </x:c>
+      <x:c r="H37" s="69" t="str">
+        <x:v>仅比配对 k-mer +0.001288；不扩展 500 标签。报告：EXP-20260930-111-hybrid-screen</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="90" customHeight="1">
+      <x:c r="A38" s="181" t="str">
+        <x:v>第九次</x:v>
+      </x:c>
+      <x:c r="B38" s="182" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C38" s="69" t="str">
+        <x:v>有效支持度分层权重：1 / 1.25 / 1.5（EXP-113）</x:v>
+      </x:c>
+      <x:c r="D38" s="69" t="str">
+        <x:v>固定尾段 1,062 样本、支持度分层 100 标签；五 seed</x:v>
+      </x:c>
+      <x:c r="E38" s="183" t="n">
+        <x:v>0.31683633498451547</x:v>
+      </x:c>
+      <x:c r="F38" s="184" t="n">
+        <x:v>0.0006093002873030889</x:v>
+      </x:c>
+      <x:c r="G38" s="184" t="n">
+        <x:v>0.803282281363617</x:v>
+      </x:c>
+      <x:c r="H38" s="69" t="str">
+        <x:v>配对增益 0.000415，2/5 seed 改善；不扩展。报告：iteration9-labelwise-weight</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="90" customHeight="1">
+      <x:c r="A39" s="181" t="str">
+        <x:v>第十次</x:v>
+      </x:c>
+      <x:c r="B39" s="182" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C39" s="69" t="str">
+        <x:v>嵌套 OOF 标签链：120k k-mer + 32 个一级 OOF 标签分数</x:v>
+      </x:c>
+      <x:c r="D39" s="69" t="str">
+        <x:v>固定尾段 1,062 样本、支持度分层 100 标签；外层/内层各两折、五 seed</x:v>
+      </x:c>
+      <x:c r="E39" s="183" t="n">
+        <x:v>0.32162199125705476</x:v>
+      </x:c>
+      <x:c r="F39" s="184" t="n">
+        <x:v>0.0013508362891496183</x:v>
+      </x:c>
+      <x:c r="G39" s="184" t="n">
+        <x:v>0.8165524381466841</x:v>
+      </x:c>
+      <x:c r="H39" s="69" t="str">
+        <x:v>比本轮一级基线 +0.005707，五 seed 全部提升；扩展到 500 标签。报告：iteration10-oof-label-chain</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="90" customHeight="1">
+      <x:c r="A40" s="181" t="str">
+        <x:v>第十一次</x:v>
+      </x:c>
+      <x:c r="B40" s="182" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C40" s="69" t="str">
+        <x:v>500 标签嵌套 OOF；120k k-mer + 64 个上下文；配对一级回退</x:v>
+      </x:c>
+      <x:c r="D40" s="69" t="str">
+        <x:v>固定尾段 1,062 样本、500 标签；外层/内层各两折、五 seed</x:v>
+      </x:c>
+      <x:c r="E40" s="183" t="n">
+        <x:v>0.3096582273393964</x:v>
+      </x:c>
+      <x:c r="F40" s="184" t="n">
+        <x:v>0.0005914280172197297</x:v>
+      </x:c>
+      <x:c r="G40" s="184" t="n">
+        <x:v>0.80573267878405</x:v>
+      </x:c>
+      <x:c r="H40" s="69" t="str">
+        <x:v>二级链 F1 0.309285，较一级下降 0.000373；停用当前配置，生产回退仍为 EXP-103。报告：iteration11-oof-label-chain-full</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="90" customHeight="1">
+      <x:c r="A41" s="181" t="str">
+        <x:v>第十二次</x:v>
+      </x:c>
+      <x:c r="B41" s="182" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C41" s="69" t="str">
+        <x:v>原始 120k k-mer + 理化性质分组 3–6-mer（权重 0.25）</x:v>
+      </x:c>
+      <x:c r="D41" s="69" t="str">
+        <x:v>固定尾段 1,062 样本、支持度分层 100 标签；五 seed</x:v>
+      </x:c>
+      <x:c r="E41" s="183" t="n">
+        <x:v>0.3172363427171758</x:v>
+      </x:c>
+      <x:c r="F41" s="184" t="n">
+        <x:v>0.0012993118180230946</x:v>
+      </x:c>
+      <x:c r="G41" s="184" t="n">
+        <x:v>0.8049595379911301</x:v>
+      </x:c>
+      <x:c r="H41" s="69" t="str">
+        <x:v>较配对原始 k-mer +0.000814；预测正例率上升，不扩展 500 标签。报告：iteration12-grouped-kmer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="90" customHeight="1">
+      <x:c r="A42" s="181" t="str">
+        <x:v>第十三次（校准诊断）</x:v>
+      </x:c>
+      <x:c r="B42" s="182" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C42" s="69" t="str">
+        <x:v>EXP-103 连续分数的支持度分层 OOF Platt 校准</x:v>
+      </x:c>
+      <x:c r="D42" s="69" t="str">
+        <x:v>固定尾段 1,062 样本、500 标签；五个校准 seed 与五个阈值 seed</x:v>
+      </x:c>
+      <x:c r="E42" s="183" t="n">
+        <x:v>0.3364394001088342</x:v>
+      </x:c>
+      <x:c r="F42" s="184" t="n">
+        <x:v>0.0017912847145465293</x:v>
+      </x:c>
+      <x:c r="G42" s="184" t="n">
+        <x:v>0.8236168289363767</x:v>
+      </x:c>
+      <x:c r="H42" s="69" t="str">
+        <x:v>正例率下降但 F1 下降 0.001943；校准不能替代排序改进，诊断结果不替换 EXP-103。报告：iteration13-prior-calibration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="90" customHeight="1">
+      <x:c r="A43" s="181" t="str">
+        <x:v>第十四次（误差诊断）</x:v>
+      </x:c>
+      <x:c r="B43" s="182" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C43" s="69" t="str">
+        <x:v>EXP-103 逐标签 classification_report、混淆矩阵与 20 条过拟合测试</x:v>
+      </x:c>
+      <x:c r="D43" s="69" t="str">
+        <x:v>固定尾段 1,062 样本、500 标签；seed-42 两折阈值交叉拟合</x:v>
+      </x:c>
+      <x:c r="E43" s="183" t="n">
+        <x:v>0.3385517949962983</x:v>
+      </x:c>
+      <x:c r="F43" s="184" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G43" s="184" t="n">
+        <x:v>0.8244919055304825</x:v>
+      </x:c>
+      <x:c r="H43" s="69" t="str">
+        <x:v>70 个标签验证正例不超过 10；identity+RF 过拟合 F1=1.0，确认瓶颈在低频表示与排序；已转 focal BCE。报告：iteration14-f1-diagnostics</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="90" customHeight="1">
+      <x:c r="A44" s="181" t="str">
+        <x:v>第十五次（ESM 审计与 EXP-117 复核）</x:v>
+      </x:c>
+      <x:c r="B44" s="182" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C44" s="69" t="str">
+        <x:v>ESM-2 35M 最后4层微调1 epoch；模型身份、标签列和窗口审计</x:v>
+      </x:c>
+      <x:c r="D44" s="69" t="str">
+        <x:v>固定尾段 1,062 样本、500 标签；与 EXP-103 相同五 seed 精确收缩阈值</x:v>
+      </x:c>
+      <x:c r="E44" s="183" t="n">
+        <x:v>0.152413970473923</x:v>
+      </x:c>
+      <x:c r="F44" s="184" t="n">
+        <x:v>0.0011034887891825274</x:v>
+      </x:c>
+      <x:c r="G44" s="184" t="n">
+        <x:v>0.6994043221362165</x:v>
+      </x:c>
+      <x:c r="H44" s="69" t="str">
+        <x:v>ESM 单源 F1 0.152414；过预测18.08%；单窗口 AUC仍仅0.702856；125多轮对照运行中，不替换103。报告：EXP-20260930-126-esm-provenance-audit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="90" customHeight="1">
+      <x:c r="A45" s="181" t="str">
+        <x:v>第十六次（EXP-125 轮数斜率）</x:v>
+      </x:c>
+      <x:c r="B45" s="182" t="d">
+        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C45" s="69" t="str">
+        <x:v>ESM-2 35M 最后4层微调；仅将 EXP-117 的 1 epoch 延长至 3 epoch</x:v>
+      </x:c>
+      <x:c r="D45" s="69" t="str">
+        <x:v>固定尾段 1,062 样本、500 标签；五 seed 精确收缩阈值、两折预测合并</x:v>
+      </x:c>
+      <x:c r="E45" s="183" t="n">
+        <x:v>0.18368143481351412</x:v>
+      </x:c>
+      <x:c r="F45" s="184" t="n">
+        <x:v>0.0015756512130494964</x:v>
+      </x:c>
+      <x:c r="G45" s="184" t="n">
+        <x:v>0.7296348412241555</x:v>
+      </x:c>
+      <x:c r="H45" s="69" t="str">
+        <x:v>AUC 0.699419→0.712810→0.729635；两段增量+0.013391/+0.016825，未趋平，优先延长训练再试池化；不替换103。报告：EXP-20260930-125-esm35-epoch-slope</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2146,6 +2952,293 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcdd2184a9564565"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f39486932a24f66"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="27" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="180" t="str">
+        <x:v>趋势图来源：公式链接登记表，分开显示不同验证口径</x:v>
+      </x:c>
+      <x:c r="B1" s="180"/>
+      <x:c r="C1" s="180"/>
+      <x:c r="D1" s="180"/>
+      <x:c r="E1" s="180"/>
+      <x:c r="F1" s="180"/>
+      <x:c r="G1" s="180"/>
+      <x:c r="H1" s="180"/>
+      <x:c r="I1" s="180"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="180" t="str">
+        <x:v>完整 500 标签目标 Macro F1</x:v>
+      </x:c>
+      <x:c r="B2" s="180" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="C2" s="180"/>
+      <x:c r="D2" s="180"/>
+      <x:c r="E2" s="180"/>
+      <x:c r="F2" s="180"/>
+      <x:c r="G2" s="180"/>
+      <x:c r="H2" s="180"/>
+      <x:c r="I2" s="180"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="190" t="str">
+        <x:v>迭代</x:v>
+      </x:c>
+      <x:c r="B4" s="190" t="str">
+        <x:v>Macro F1</x:v>
+      </x:c>
+      <x:c r="C4" s="190" t="str">
+        <x:v>目标 0.5</x:v>
+      </x:c>
+      <x:c r="E4" s="190" t="str">
+        <x:v>筛选实验</x:v>
+      </x:c>
+      <x:c r="F4" s="190" t="str">
+        <x:v>Macro F1</x:v>
+      </x:c>
+      <x:c r="H4" s="190" t="str">
+        <x:v>历史随机验证</x:v>
+      </x:c>
+      <x:c r="I4" s="190" t="str">
+        <x:v>Macro F1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:f>'迭代趋势'!A8</x:f>
+        <x:v>第三次</x:v>
+      </x:c>
+      <x:c r="B5" s="185" t="n">
+        <x:f>'迭代趋势'!E8</x:f>
+        <x:v>0.3215169269432081</x:v>
+      </x:c>
+      <x:c r="C5" t="n">
+        <x:f>$B$2</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:f>'迭代趋势'!A37</x:f>
+        <x:v>联合特征筛选（111）</x:v>
+      </x:c>
+      <x:c r="F5" s="185" t="n">
+        <x:f>'迭代趋势'!E37</x:f>
+        <x:v>0.3184272015000932</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:f>'迭代趋势'!A6</x:f>
+        <x:v>第一次</x:v>
+      </x:c>
+      <x:c r="I5" s="185" t="n">
+        <x:f>'迭代趋势'!E6</x:f>
+        <x:v>0.3799564929582331</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:f>'迭代趋势'!A9</x:f>
+        <x:v>第四次</x:v>
+      </x:c>
+      <x:c r="B6" s="185" t="n">
+        <x:f>'迭代趋势'!E9</x:f>
+        <x:v>0.32419172996031437</x:v>
+      </x:c>
+      <x:c r="C6" t="n">
+        <x:f>$B$2</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:f>'迭代趋势'!A38</x:f>
+        <x:v>第九次</x:v>
+      </x:c>
+      <x:c r="F6" s="185" t="n">
+        <x:f>'迭代趋势'!E38</x:f>
+        <x:v>0.31683633498451547</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:f>'迭代趋势'!A7</x:f>
+        <x:v>第二次</x:v>
+      </x:c>
+      <x:c r="I6" s="185" t="n">
+        <x:f>'迭代趋势'!E7</x:f>
+        <x:v>0.24636956251082398</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:f>'迭代趋势'!A10</x:f>
+        <x:v>第五次</x:v>
+      </x:c>
+      <x:c r="B7" s="185" t="n">
+        <x:f>'迭代趋势'!E10</x:f>
+        <x:v>0.3351783934801672</x:v>
+      </x:c>
+      <x:c r="C7" t="n">
+        <x:f>$B$2</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:f>'迭代趋势'!A39</x:f>
+        <x:v>第十次</x:v>
+      </x:c>
+      <x:c r="F7" s="185" t="n">
+        <x:f>'迭代趋势'!E39</x:f>
+        <x:v>0.32162199125705476</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:f>'迭代趋势'!A11</x:f>
+        <x:v>第六次</x:v>
+      </x:c>
+      <x:c r="B8" s="185" t="n">
+        <x:f>'迭代趋势'!E11</x:f>
+        <x:v>0.3242434409979672</x:v>
+      </x:c>
+      <x:c r="C8" t="n">
+        <x:f>$B$2</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:f>'迭代趋势'!A41</x:f>
+        <x:v>第十二次</x:v>
+      </x:c>
+      <x:c r="F8" s="185" t="n">
+        <x:f>'迭代趋势'!E41</x:f>
+        <x:v>0.3172363427171758</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:f>'迭代趋势'!A35</x:f>
+        <x:v>第七次（产物复核）</x:v>
+      </x:c>
+      <x:c r="B9" s="185" t="n">
+        <x:f>'迭代趋势'!E35</x:f>
+        <x:v>0.32430998512037634</x:v>
+      </x:c>
+      <x:c r="C9" t="n">
+        <x:f>$B$2</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:f>'迭代趋势'!A36</x:f>
+        <x:v>第八次</x:v>
+      </x:c>
+      <x:c r="B10" s="185" t="n">
+        <x:f>'迭代趋势'!E36</x:f>
+        <x:v>0.3382479496821853</x:v>
+      </x:c>
+      <x:c r="C10" t="n">
+        <x:f>$B$2</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:f>'迭代趋势'!A40</x:f>
+        <x:v>第十一次</x:v>
+      </x:c>
+      <x:c r="B11" s="185" t="n">
+        <x:f>'迭代趋势'!E40</x:f>
+        <x:v>0.3096582273393964</x:v>
+      </x:c>
+      <x:c r="C11" t="n">
+        <x:f>$B$2</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:f>'迭代趋势'!A42</x:f>
+        <x:v>第十三次（校准诊断）</x:v>
+      </x:c>
+      <x:c r="B12" s="185" t="n">
+        <x:f>'迭代趋势'!E42</x:f>
+        <x:v>0.3364394001088342</x:v>
+      </x:c>
+      <x:c r="C12" t="n">
+        <x:f>$B$2</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:f>'迭代趋势'!A43</x:f>
+        <x:v>第十四次（误差诊断）</x:v>
+      </x:c>
+      <x:c r="B13" s="185" t="n">
+        <x:f>'迭代趋势'!E43</x:f>
+        <x:v>0.3385517949962983</x:v>
+      </x:c>
+      <x:c r="C13" t="n">
+        <x:f>$B$2</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:f>'迭代趋势'!A44</x:f>
+        <x:v>第十五次（ESM 审计与 EXP-117 复核）</x:v>
+      </x:c>
+      <x:c r="B14" s="185" t="n">
+        <x:f>'迭代趋势'!E44</x:f>
+        <x:v>0.152413970473923</x:v>
+      </x:c>
+      <x:c r="C14" t="n">
+        <x:f>$B$2</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:f>'迭代趋势'!A45</x:f>
+        <x:v>第十六次（EXP-125 轮数斜率）</x:v>
+      </x:c>
+      <x:c r="B15" s="185" t="n">
+        <x:f>'迭代趋势'!E45</x:f>
+        <x:v>0.18368143481351412</x:v>
+      </x:c>
+      <x:c r="C15" t="n">
+        <x:f>$B$2</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>尾段图只包含 500 标签结果；方法与校准协议仍会变化，不能当作线上成绩。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>100 标签筛选单列；随机验证历史单列，不与尾段成绩连接。</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>